<commit_message>
update end device gps
</commit_message>
<xml_diff>
--- a/3_N4_Armazenamento/Parametros/Pacote_DL_UL.xlsx
+++ b/3_N4_Armazenamento/Parametros/Pacote_DL_UL.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\Pos-Doc\Frameworks\Artigo\Framework_DL_UL_MQTT_PAR\LoRa_Survey_MQTT_Net_GPS\LoRa_Survey_MQTT_Nodes\3_N4_Armazenamento\Parametros\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\Pos-Doc\Frameworks\Artigo\Framework_DL_UL_MQTT_PAR\LoRa_Survey_MQTT_Net_GPS\LoRa_MQTT_Multiple_Nodes\3_N4_Armazenamento\Parametros\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="20 Bytes" sheetId="1" r:id="rId1"/>
     <sheet name="30 Bytes" sheetId="2" r:id="rId2"/>
+    <sheet name="DL20-UL30" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="49">
   <si>
     <t>UL_B</t>
   </si>
@@ -657,14 +658,14 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -959,17 +960,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="3"/>
       <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1"/>
+      <c r="G1" s="3"/>
       <c r="H1" t="s">
         <v>1</v>
       </c>
@@ -1106,7 +1107,7 @@
       <c r="H6">
         <v>26</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="1" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1132,7 +1133,7 @@
       <c r="H7">
         <v>27</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="1" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1158,7 +1159,7 @@
       <c r="H8">
         <v>28</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="1" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1184,7 +1185,7 @@
       <c r="H9">
         <v>29</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="1" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1213,7 +1214,7 @@
       <c r="I10" t="s">
         <v>8</v>
       </c>
-      <c r="L10" s="3"/>
+      <c r="L10" s="2"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1237,7 +1238,7 @@
       <c r="H11">
         <v>31</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" s="1" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1266,7 +1267,7 @@
       <c r="I12" t="s">
         <v>7</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="L12" s="1" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1289,7 +1290,7 @@
       <c r="H13">
         <v>33</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="L13" s="1" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1312,7 +1313,7 @@
       <c r="H14">
         <v>34</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="L14" s="1" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1335,7 +1336,7 @@
       <c r="H15">
         <v>35</v>
       </c>
-      <c r="L15" s="3"/>
+      <c r="L15" s="2"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1356,7 +1357,7 @@
       <c r="H16">
         <v>36</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="L16" s="1" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1379,7 +1380,7 @@
       <c r="H17">
         <v>37</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="L17" s="1" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1402,7 +1403,7 @@
       <c r="H18">
         <v>38</v>
       </c>
-      <c r="L18" s="2" t="s">
+      <c r="L18" s="1" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1425,7 +1426,7 @@
       <c r="H19">
         <v>39</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="L19" s="1" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1530,17 +1531,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="3"/>
       <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1"/>
+      <c r="G1" s="3"/>
       <c r="H1" t="s">
         <v>1</v>
       </c>
@@ -2248,6 +2249,663 @@
       </c>
       <c r="H31">
         <v>61</v>
+      </c>
+      <c r="I31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="F1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.42578125" customWidth="1"/>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.140625" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" customWidth="1"/>
+    <col min="7" max="7" width="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="31.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="3"/>
+      <c r="H1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>22</v>
+      </c>
+      <c r="I2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
+        <v>24</v>
+      </c>
+      <c r="I4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>6</v>
+      </c>
+      <c r="H8">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>7</v>
+      </c>
+      <c r="H9">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>8</v>
+      </c>
+      <c r="H10">
+        <v>30</v>
+      </c>
+      <c r="I10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>9</v>
+      </c>
+      <c r="H11">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>10</v>
+      </c>
+      <c r="H12">
+        <v>32</v>
+      </c>
+      <c r="I12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>11</v>
+      </c>
+      <c r="H13">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14">
+        <v>12</v>
+      </c>
+      <c r="C14">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>12</v>
+      </c>
+      <c r="H14">
+        <v>34</v>
+      </c>
+      <c r="I14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15">
+        <v>13</v>
+      </c>
+      <c r="C15">
+        <v>15</v>
+      </c>
+      <c r="F15" t="s">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>13</v>
+      </c>
+      <c r="H15">
+        <v>35</v>
+      </c>
+      <c r="I15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16">
+        <v>14</v>
+      </c>
+      <c r="C16">
+        <v>16</v>
+      </c>
+      <c r="F16" t="s">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>14</v>
+      </c>
+      <c r="H16">
+        <v>36</v>
+      </c>
+      <c r="I16" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
+      <c r="C17">
+        <v>17</v>
+      </c>
+      <c r="F17" t="s">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>15</v>
+      </c>
+      <c r="H17">
+        <v>37</v>
+      </c>
+      <c r="I17" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18">
+        <v>16</v>
+      </c>
+      <c r="C18">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>16</v>
+      </c>
+      <c r="H18">
+        <v>38</v>
+      </c>
+      <c r="I18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19">
+        <v>17</v>
+      </c>
+      <c r="C19">
+        <v>19</v>
+      </c>
+      <c r="F19" t="s">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>17</v>
+      </c>
+      <c r="H19">
+        <v>39</v>
+      </c>
+      <c r="I19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20">
+        <v>18</v>
+      </c>
+      <c r="C20">
+        <v>20</v>
+      </c>
+      <c r="F20" t="s">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>18</v>
+      </c>
+      <c r="H20">
+        <v>40</v>
+      </c>
+      <c r="I20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21">
+        <v>19</v>
+      </c>
+      <c r="C21">
+        <v>21</v>
+      </c>
+      <c r="F21" t="s">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>19</v>
+      </c>
+      <c r="H21">
+        <v>41</v>
+      </c>
+      <c r="I21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>20</v>
+      </c>
+      <c r="H22">
+        <v>42</v>
+      </c>
+      <c r="I22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>21</v>
+      </c>
+      <c r="H23">
+        <v>43</v>
+      </c>
+      <c r="I23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F24" t="s">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>22</v>
+      </c>
+      <c r="H24">
+        <v>44</v>
+      </c>
+      <c r="I24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>23</v>
+      </c>
+      <c r="H25">
+        <v>45</v>
+      </c>
+      <c r="I25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F26" t="s">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>24</v>
+      </c>
+      <c r="H26">
+        <v>46</v>
+      </c>
+      <c r="I26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F27" t="s">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>25</v>
+      </c>
+      <c r="H27">
+        <v>47</v>
+      </c>
+      <c r="I27" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>26</v>
+      </c>
+      <c r="H28">
+        <v>48</v>
+      </c>
+      <c r="I28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F29" t="s">
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <v>27</v>
+      </c>
+      <c r="H29">
+        <v>49</v>
+      </c>
+      <c r="I29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F30" t="s">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>28</v>
+      </c>
+      <c r="H30">
+        <v>50</v>
+      </c>
+      <c r="I30" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F31" t="s">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>29</v>
+      </c>
+      <c r="H31">
+        <v>51</v>
       </c>
       <c r="I31" t="s">
         <v>31</v>

</xml_diff>